<commit_message>
Update summer baseline and max_rank calculation
</commit_message>
<xml_diff>
--- a/data/hdu_contest.xlsx
+++ b/data/hdu_contest.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3840" yWindow="3840" windowWidth="23040" windowHeight="12072" tabRatio="600" firstSheet="0" activeTab="9" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25600" windowHeight="10480" tabRatio="600" firstSheet="0" activeTab="9" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="hdu1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="hdu2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="hdu3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="hdu4" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="hdu5" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="hdu6" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="hdu7" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="hdu8" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="hdu9" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="hdu10" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu6" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu7" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu8" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu9" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hdu10" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="23">
     <font>
       <name val="宋体"/>
-      <family val="2"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -43,12 +43,164 @@
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -61,8 +213,194 @@
         <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -70,18 +408,311 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -434,7 +1065,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -444,8 +1074,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -481,6 +1111,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>得分</t>
         </is>
       </c>
@@ -503,10 +1138,13 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>34.97</v>
+        <v>791</v>
+      </c>
+      <c r="G2" t="n">
+        <v>33.54</v>
       </c>
     </row>
     <row r="3">
@@ -527,10 +1165,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>31.43</v>
+        <v>791</v>
+      </c>
+      <c r="G3" t="n">
+        <v>31.8</v>
       </c>
     </row>
     <row r="4">
@@ -551,10 +1192,13 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
-        <v>31.89</v>
+        <v>791</v>
+      </c>
+      <c r="G4" t="n">
+        <v>32.03</v>
       </c>
     </row>
     <row r="5">
@@ -575,10 +1219,13 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
-        <v>22.86</v>
+        <v>791</v>
+      </c>
+      <c r="G5" t="n">
+        <v>27.59</v>
       </c>
     </row>
     <row r="6">
@@ -599,10 +1246,13 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
-        <v>23.54</v>
+        <v>791</v>
+      </c>
+      <c r="G6" t="n">
+        <v>27.93</v>
       </c>
     </row>
     <row r="7">
@@ -623,10 +1273,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>791</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.21</v>
       </c>
     </row>
     <row r="8">
@@ -647,10 +1300,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>59.57</v>
+        <v>791</v>
+      </c>
+      <c r="G8" t="n">
+        <v>49.73</v>
       </c>
     </row>
     <row r="9">
@@ -671,10 +1327,13 @@
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>29.71</v>
+        <v>791</v>
+      </c>
+      <c r="G9" t="n">
+        <v>30.96</v>
       </c>
     </row>
     <row r="10">
@@ -695,10 +1354,13 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>791</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.37</v>
       </c>
     </row>
     <row r="11">
@@ -719,10 +1381,13 @@
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>0.51</v>
+        <v>791</v>
+      </c>
+      <c r="G11" t="n">
+        <v>12.52</v>
       </c>
     </row>
     <row r="12">
@@ -743,10 +1408,13 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>791</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.59</v>
       </c>
     </row>
     <row r="13">
@@ -767,10 +1435,13 @@
         <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F13" t="n">
-        <v>35.2</v>
+        <v>791</v>
+      </c>
+      <c r="G13" t="n">
+        <v>33.66</v>
       </c>
     </row>
     <row r="14">
@@ -791,10 +1462,13 @@
         <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
-        <v>60.86</v>
+        <v>791</v>
+      </c>
+      <c r="G14" t="n">
+        <v>50.36</v>
       </c>
     </row>
   </sheetData>
@@ -809,8 +1483,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -844,7 +1518,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -868,10 +1547,13 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>23</v>
+        <v>652</v>
+      </c>
+      <c r="G2" t="n">
+        <v>25.88</v>
       </c>
     </row>
     <row r="3">
@@ -892,10 +1574,13 @@
         <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>29.56</v>
+        <v>652</v>
+      </c>
+      <c r="G3" t="n">
+        <v>32.44</v>
       </c>
     </row>
     <row r="4">
@@ -916,10 +1601,13 @@
         <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>36.33</v>
+        <v>652</v>
+      </c>
+      <c r="G4" t="n">
+        <v>37.19</v>
       </c>
     </row>
     <row r="5">
@@ -939,9 +1627,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
+        <v>652</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -963,10 +1654,13 @@
         <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>35.02</v>
+        <v>652</v>
+      </c>
+      <c r="G6" t="n">
+        <v>36.27</v>
       </c>
     </row>
     <row r="7">
@@ -987,10 +1681,13 @@
         <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>32.51</v>
+        <v>652</v>
+      </c>
+      <c r="G7" t="n">
+        <v>34.51</v>
       </c>
     </row>
     <row r="8">
@@ -1011,10 +1708,13 @@
         <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>56.58</v>
+        <v>652</v>
+      </c>
+      <c r="G8" t="n">
+        <v>55.32</v>
       </c>
     </row>
     <row r="9">
@@ -1035,10 +1735,13 @@
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>35.78</v>
+        <v>652</v>
+      </c>
+      <c r="G9" t="n">
+        <v>36.81</v>
       </c>
     </row>
     <row r="10">
@@ -1059,10 +1762,13 @@
         <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>11.91</v>
+        <v>652</v>
+      </c>
+      <c r="G10" t="n">
+        <v>18.09</v>
       </c>
     </row>
     <row r="11">
@@ -1083,10 +1789,13 @@
         <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>15</v>
+        <v>652</v>
+      </c>
+      <c r="G11" t="n">
+        <v>20.26</v>
       </c>
     </row>
     <row r="12">
@@ -1107,10 +1816,13 @@
         <v>5</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>13.73</v>
+        <v>652</v>
+      </c>
+      <c r="G12" t="n">
+        <v>19.36</v>
       </c>
     </row>
     <row r="13">
@@ -1131,10 +1843,13 @@
         <v>6</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>35.56</v>
+        <v>652</v>
+      </c>
+      <c r="G13" t="n">
+        <v>36.66</v>
       </c>
     </row>
     <row r="14">
@@ -1155,10 +1870,13 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>652</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.29</v>
       </c>
     </row>
   </sheetData>
@@ -1173,8 +1891,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1208,7 +1926,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -1232,10 +1955,13 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>26.9</v>
+        <v>684</v>
+      </c>
+      <c r="G2" t="n">
+        <v>26.49</v>
       </c>
     </row>
     <row r="3">
@@ -1256,10 +1982,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>30.6</v>
+        <v>684</v>
+      </c>
+      <c r="G3" t="n">
+        <v>28.65</v>
       </c>
     </row>
     <row r="4">
@@ -1280,10 +2009,13 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>43</v>
+        <v>684</v>
+      </c>
+      <c r="G4" t="n">
+        <v>38.6</v>
       </c>
     </row>
     <row r="5">
@@ -1304,10 +2036,13 @@
         <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>63.15</v>
+        <v>684</v>
+      </c>
+      <c r="G5" t="n">
+        <v>53.07</v>
       </c>
     </row>
     <row r="6">
@@ -1328,10 +2063,13 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>33.1</v>
+        <v>684</v>
+      </c>
+      <c r="G6" t="n">
+        <v>30.12</v>
       </c>
     </row>
     <row r="7">
@@ -1352,10 +2090,13 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>9.449999999999999</v>
+        <v>684</v>
+      </c>
+      <c r="G7" t="n">
+        <v>13.6</v>
       </c>
     </row>
     <row r="8">
@@ -1376,10 +2117,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>44</v>
+        <v>684</v>
+      </c>
+      <c r="G8" t="n">
+        <v>39.18</v>
       </c>
     </row>
     <row r="9">
@@ -1400,10 +2144,13 @@
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>29.8</v>
+        <v>684</v>
+      </c>
+      <c r="G9" t="n">
+        <v>28.19</v>
       </c>
     </row>
     <row r="10">
@@ -1424,10 +2171,13 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>10.05</v>
+        <v>684</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13.95</v>
       </c>
     </row>
     <row r="11">
@@ -1448,10 +2198,13 @@
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>9.529999999999999</v>
+        <v>684</v>
+      </c>
+      <c r="G11" t="n">
+        <v>13.64</v>
       </c>
     </row>
     <row r="12">
@@ -1472,10 +2225,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>684</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.33</v>
       </c>
     </row>
     <row r="13">
@@ -1496,10 +2252,13 @@
         <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>3.55</v>
+        <v>684</v>
+      </c>
+      <c r="G13" t="n">
+        <v>7.46</v>
       </c>
     </row>
     <row r="14">
@@ -1520,10 +2279,13 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F14" t="n">
-        <v>0.75</v>
+        <v>684</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.82</v>
       </c>
     </row>
   </sheetData>
@@ -1537,8 +2299,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1572,7 +2334,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -1595,9 +2362,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
+        <v>699</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1619,10 +2389,13 @@
         <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>39.2</v>
+        <v>699</v>
+      </c>
+      <c r="G3" t="n">
+        <v>35.26</v>
       </c>
     </row>
     <row r="4">
@@ -1643,10 +2416,13 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>20.22</v>
+        <v>699</v>
+      </c>
+      <c r="G4" t="n">
+        <v>22.71</v>
       </c>
     </row>
     <row r="5">
@@ -1667,10 +2443,13 @@
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>66.73</v>
+        <v>699</v>
+      </c>
+      <c r="G5" t="n">
+        <v>52.41</v>
       </c>
     </row>
     <row r="6">
@@ -1691,10 +2470,13 @@
         <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>31.07</v>
+        <v>699</v>
+      </c>
+      <c r="G6" t="n">
+        <v>30.9</v>
       </c>
     </row>
     <row r="7">
@@ -1715,10 +2497,13 @@
         <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>15.22</v>
+        <v>699</v>
+      </c>
+      <c r="G7" t="n">
+        <v>20.03</v>
       </c>
     </row>
     <row r="8">
@@ -1739,10 +2524,13 @@
         <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>42.67</v>
+        <v>699</v>
+      </c>
+      <c r="G8" t="n">
+        <v>37.12</v>
       </c>
     </row>
     <row r="9">
@@ -1763,10 +2551,13 @@
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>22.33</v>
+        <v>699</v>
+      </c>
+      <c r="G9" t="n">
+        <v>23.84</v>
       </c>
     </row>
     <row r="10">
@@ -1787,10 +2578,13 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>699</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5.44</v>
       </c>
     </row>
     <row r="11">
@@ -1811,10 +2605,13 @@
         <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>20.78</v>
+        <v>699</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23.01</v>
       </c>
     </row>
     <row r="12">
@@ -1835,10 +2632,13 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>699</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.11</v>
       </c>
     </row>
     <row r="13">
@@ -1859,10 +2659,13 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>699</v>
+      </c>
+      <c r="G13" t="n">
+        <v>18.3</v>
       </c>
     </row>
     <row r="14">
@@ -1883,10 +2686,13 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>699</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.74</v>
       </c>
     </row>
   </sheetData>
@@ -1901,8 +2707,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1936,7 +2742,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -1959,9 +2770,12 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
+        <v>729</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1983,10 +2797,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>22.4</v>
+        <v>729</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20.71</v>
       </c>
     </row>
     <row r="4">
@@ -2007,10 +2824,13 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>43.5</v>
+        <v>729</v>
+      </c>
+      <c r="G4" t="n">
+        <v>32.98</v>
       </c>
     </row>
     <row r="5">
@@ -2031,10 +2851,13 @@
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>81.2</v>
+        <v>729</v>
+      </c>
+      <c r="G5" t="n">
+        <v>55.45</v>
       </c>
     </row>
     <row r="6">
@@ -2055,10 +2878,13 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>17.3</v>
+        <v>729</v>
+      </c>
+      <c r="G6" t="n">
+        <v>18.38</v>
       </c>
     </row>
     <row r="7">
@@ -2079,10 +2905,13 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>7.2</v>
+        <v>729</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.15</v>
       </c>
     </row>
     <row r="8">
@@ -2103,10 +2932,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>45.5</v>
+        <v>729</v>
+      </c>
+      <c r="G8" t="n">
+        <v>33.89</v>
       </c>
     </row>
     <row r="9">
@@ -2127,10 +2959,13 @@
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>59.4</v>
+        <v>729</v>
+      </c>
+      <c r="G9" t="n">
+        <v>42.87</v>
       </c>
     </row>
     <row r="10">
@@ -2151,10 +2986,13 @@
         <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>15</v>
+        <v>729</v>
+      </c>
+      <c r="G10" t="n">
+        <v>17.33</v>
       </c>
     </row>
     <row r="11">
@@ -2175,10 +3013,13 @@
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>5.47</v>
+        <v>729</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.36</v>
       </c>
     </row>
     <row r="12">
@@ -2199,10 +3040,13 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0.83</v>
+        <v>729</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8.23</v>
       </c>
     </row>
     <row r="13">
@@ -2223,10 +3067,13 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>38.5</v>
+        <v>729</v>
+      </c>
+      <c r="G13" t="n">
+        <v>30.69</v>
       </c>
     </row>
     <row r="14">
@@ -2247,10 +3094,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>729</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.19</v>
       </c>
     </row>
   </sheetData>
@@ -2265,8 +3115,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2300,7 +3150,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -2324,10 +3179,13 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>20.4</v>
+        <v>757</v>
+      </c>
+      <c r="G2" t="n">
+        <v>17.47</v>
       </c>
     </row>
     <row r="3">
@@ -2348,10 +3206,13 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>18.15</v>
+        <v>757</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16.48</v>
       </c>
     </row>
     <row r="4">
@@ -2372,10 +3233,13 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>48.62</v>
+        <v>757</v>
+      </c>
+      <c r="G4" t="n">
+        <v>35.56</v>
       </c>
     </row>
     <row r="5">
@@ -2396,10 +3260,13 @@
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>53.5</v>
+        <v>757</v>
+      </c>
+      <c r="G5" t="n">
+        <v>37.7</v>
       </c>
     </row>
     <row r="6">
@@ -2420,10 +3287,13 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>11.18</v>
+        <v>757</v>
+      </c>
+      <c r="G6" t="n">
+        <v>13.41</v>
       </c>
     </row>
     <row r="7">
@@ -2444,10 +3314,13 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>12.97</v>
+        <v>757</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14.2</v>
       </c>
     </row>
     <row r="8">
@@ -2468,10 +3341,13 @@
         <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>17.25</v>
+        <v>757</v>
+      </c>
+      <c r="G8" t="n">
+        <v>16.08</v>
       </c>
     </row>
     <row r="9">
@@ -2492,10 +3368,13 @@
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>33.5</v>
+        <v>757</v>
+      </c>
+      <c r="G9" t="n">
+        <v>26.07</v>
       </c>
     </row>
     <row r="10">
@@ -2516,10 +3395,13 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>757</v>
+      </c>
+      <c r="G10" t="n">
+        <v>8.220000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2540,10 +3422,13 @@
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>757</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9.81</v>
       </c>
     </row>
     <row r="12">
@@ -2564,10 +3449,13 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>757</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.21</v>
       </c>
     </row>
     <row r="13">
@@ -2588,10 +3476,13 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>16.35</v>
+        <v>757</v>
+      </c>
+      <c r="G13" t="n">
+        <v>15.69</v>
       </c>
     </row>
     <row r="14">
@@ -2611,9 +3502,12 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
+        <v>757</v>
+      </c>
+      <c r="G14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2629,8 +3523,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2664,7 +3558,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -2688,10 +3587,13 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>41.11</v>
+        <v>713</v>
+      </c>
+      <c r="G2" t="n">
+        <v>34.07</v>
       </c>
     </row>
     <row r="3">
@@ -2712,10 +3614,13 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>8.33</v>
+        <v>713</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11.85</v>
       </c>
     </row>
     <row r="4">
@@ -2736,10 +3641,13 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>40.44</v>
+        <v>713</v>
+      </c>
+      <c r="G4" t="n">
+        <v>33.72</v>
       </c>
     </row>
     <row r="5">
@@ -2760,10 +3668,13 @@
         <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>54.4</v>
+        <v>713</v>
+      </c>
+      <c r="G5" t="n">
+        <v>43.55</v>
       </c>
     </row>
     <row r="6">
@@ -2784,10 +3695,13 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>20.27</v>
+        <v>713</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20.62</v>
       </c>
     </row>
     <row r="7">
@@ -2808,10 +3722,13 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>6.4</v>
+        <v>713</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10.83</v>
       </c>
     </row>
     <row r="8">
@@ -2832,10 +3749,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>39.56</v>
+        <v>713</v>
+      </c>
+      <c r="G8" t="n">
+        <v>33.25</v>
       </c>
     </row>
     <row r="9">
@@ -2856,10 +3776,13 @@
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>40.56</v>
+        <v>713</v>
+      </c>
+      <c r="G9" t="n">
+        <v>33.78</v>
       </c>
     </row>
     <row r="10">
@@ -2880,10 +3803,13 @@
         <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>16.98</v>
+        <v>713</v>
+      </c>
+      <c r="G10" t="n">
+        <v>18.89</v>
       </c>
     </row>
     <row r="11">
@@ -2904,10 +3830,13 @@
         <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>3.67</v>
+        <v>713</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="12">
@@ -2928,10 +3857,13 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>713</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.46</v>
       </c>
     </row>
     <row r="13">
@@ -2952,10 +3884,13 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>39.11</v>
+        <v>713</v>
+      </c>
+      <c r="G13" t="n">
+        <v>33.02</v>
       </c>
     </row>
     <row r="14">
@@ -2976,10 +3911,13 @@
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>17.96</v>
+        <v>713</v>
+      </c>
+      <c r="G14" t="n">
+        <v>19.4</v>
       </c>
     </row>
   </sheetData>
@@ -2994,8 +3932,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3029,7 +3967,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -3053,10 +3996,13 @@
         <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>46.13</v>
+        <v>726</v>
+      </c>
+      <c r="G2" t="n">
+        <v>42.98</v>
       </c>
     </row>
     <row r="3">
@@ -3077,10 +4023,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>9.779999999999999</v>
+        <v>726</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16.83</v>
       </c>
     </row>
     <row r="4">
@@ -3101,10 +4050,13 @@
         <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>41.07</v>
+        <v>726</v>
+      </c>
+      <c r="G4" t="n">
+        <v>40.12</v>
       </c>
     </row>
     <row r="5">
@@ -3125,10 +4077,13 @@
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>67.2</v>
+        <v>726</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57.68</v>
       </c>
     </row>
     <row r="6">
@@ -3149,10 +4104,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>27.56</v>
+        <v>726</v>
+      </c>
+      <c r="G6" t="n">
+        <v>29.68</v>
       </c>
     </row>
     <row r="7">
@@ -3173,10 +4131,13 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>6.49</v>
+        <v>726</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14.98</v>
       </c>
     </row>
     <row r="8">
@@ -3197,10 +4158,13 @@
         <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>43.07</v>
+        <v>726</v>
+      </c>
+      <c r="G8" t="n">
+        <v>41.25</v>
       </c>
     </row>
     <row r="9">
@@ -3221,10 +4185,13 @@
         <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>62.07</v>
+        <v>726</v>
+      </c>
+      <c r="G9" t="n">
+        <v>54.78</v>
       </c>
     </row>
     <row r="10">
@@ -3245,10 +4212,13 @@
         <v>4</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F10" t="n">
-        <v>10.4</v>
+        <v>726</v>
+      </c>
+      <c r="G10" t="n">
+        <v>17.18</v>
       </c>
     </row>
     <row r="11">
@@ -3269,10 +4239,13 @@
         <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
-        <v>6.67</v>
+        <v>726</v>
+      </c>
+      <c r="G11" t="n">
+        <v>15.08</v>
       </c>
     </row>
     <row r="12">
@@ -3293,10 +4266,13 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>726</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7.33</v>
       </c>
     </row>
     <row r="13">
@@ -3317,10 +4293,13 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
-        <v>26.33</v>
+        <v>726</v>
+      </c>
+      <c r="G13" t="n">
+        <v>28.99</v>
       </c>
     </row>
     <row r="14">
@@ -3341,10 +4320,13 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>726</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.96</v>
       </c>
     </row>
   </sheetData>
@@ -3359,8 +4341,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3394,7 +4376,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -3418,10 +4405,13 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>17.5</v>
+        <v>718</v>
+      </c>
+      <c r="G2" t="n">
+        <v>22.81</v>
       </c>
     </row>
     <row r="3">
@@ -3442,10 +4432,13 @@
         <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>9.6</v>
+        <v>718</v>
+      </c>
+      <c r="G3" t="n">
+        <v>18.22</v>
       </c>
     </row>
     <row r="4">
@@ -3466,10 +4459,13 @@
         <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>39.12</v>
+        <v>718</v>
+      </c>
+      <c r="G4" t="n">
+        <v>37.88</v>
       </c>
     </row>
     <row r="5">
@@ -3490,10 +4486,13 @@
         <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>70.08</v>
+        <v>718</v>
+      </c>
+      <c r="G5" t="n">
+        <v>60.91</v>
       </c>
     </row>
     <row r="6">
@@ -3514,10 +4513,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>16.8</v>
+        <v>718</v>
+      </c>
+      <c r="G6" t="n">
+        <v>22.4</v>
       </c>
     </row>
     <row r="7">
@@ -3538,10 +4540,13 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>3.28</v>
+        <v>718</v>
+      </c>
+      <c r="G7" t="n">
+        <v>12.02</v>
       </c>
     </row>
     <row r="8">
@@ -3562,10 +4567,13 @@
         <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>56.84</v>
+        <v>718</v>
+      </c>
+      <c r="G8" t="n">
+        <v>50.7</v>
       </c>
     </row>
     <row r="9">
@@ -3586,10 +4594,13 @@
         <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>68.95999999999999</v>
+        <v>718</v>
+      </c>
+      <c r="G9" t="n">
+        <v>60.26</v>
       </c>
     </row>
     <row r="10">
@@ -3610,10 +4621,13 @@
         <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>18.8</v>
+        <v>718</v>
+      </c>
+      <c r="G10" t="n">
+        <v>23.56</v>
       </c>
     </row>
     <row r="11">
@@ -3634,10 +4648,13 @@
         <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>10.1</v>
+        <v>718</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18.51</v>
       </c>
     </row>
     <row r="12">
@@ -3658,10 +4675,13 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>718</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.11</v>
       </c>
     </row>
     <row r="13">
@@ -3682,10 +4702,13 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>23.5</v>
+        <v>718</v>
+      </c>
+      <c r="G13" t="n">
+        <v>26.29</v>
       </c>
     </row>
     <row r="14">
@@ -3706,10 +4729,13 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>718</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3724,8 +4750,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3759,7 +4785,12 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>得分</t>
         </is>
@@ -3783,10 +4814,13 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>16.62</v>
+        <v>689</v>
+      </c>
+      <c r="G2" t="n">
+        <v>19.84</v>
       </c>
     </row>
     <row r="3">
@@ -3807,10 +4841,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>16.36</v>
+        <v>689</v>
+      </c>
+      <c r="G3" t="n">
+        <v>19.69</v>
       </c>
     </row>
     <row r="4">
@@ -3831,10 +4868,13 @@
         <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>58.64</v>
+        <v>689</v>
+      </c>
+      <c r="G4" t="n">
+        <v>52.28</v>
       </c>
     </row>
     <row r="5">
@@ -3854,9 +4894,12 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
+        <v>689</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3878,10 +4921,13 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>11.82</v>
+        <v>689</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16.99</v>
       </c>
     </row>
     <row r="7">
@@ -3902,10 +4948,13 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>2.4</v>
+        <v>689</v>
+      </c>
+      <c r="G7" t="n">
+        <v>8.91</v>
       </c>
     </row>
     <row r="8">
@@ -3926,10 +4975,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>23.67</v>
+        <v>689</v>
+      </c>
+      <c r="G8" t="n">
+        <v>26.52</v>
       </c>
     </row>
     <row r="9">
@@ -3950,10 +5002,13 @@
         <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>62.69</v>
+        <v>689</v>
+      </c>
+      <c r="G9" t="n">
+        <v>54.68</v>
       </c>
     </row>
     <row r="10">
@@ -3974,10 +5029,13 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>689</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.98</v>
       </c>
     </row>
     <row r="11">
@@ -3998,10 +5056,13 @@
         <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
-        <v>15.11</v>
+        <v>689</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18.95</v>
       </c>
     </row>
     <row r="12">
@@ -4022,10 +5083,13 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>689</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6.85</v>
       </c>
     </row>
     <row r="13">
@@ -4046,10 +5110,13 @@
         <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
-        <v>15.82</v>
+        <v>689</v>
+      </c>
+      <c r="G13" t="n">
+        <v>19.37</v>
       </c>
     </row>
     <row r="14">
@@ -4070,10 +5137,13 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>689</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>